<commit_message>
Add training logs and results from Kaggle Chrome
</commit_message>
<xml_diff>
--- a/results/bang_tong_hop_luan_van.xlsx
+++ b/results/bang_tong_hop_luan_van.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ST-WaveFormer</t>
+          <t>CatBoost (Module A)</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -501,54 +501,54 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>15.350 ± 0.310</t>
+          <t>8.425 ± 0.023</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>[15.117, 15.584]</t>
+          <t>[8.408, 8.442]</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>65.385 ± 1.114</t>
+          <t>55.739 ± 0.053</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[64.545, 66.226]</t>
+          <t>[55.699, 55.779]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.1239 ± 0.0013</t>
+          <t>0.0918 ± 0.0001</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.1470</t>
+          <t>0.0807</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1837.9218</t>
+          <t>0.3089</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>3.64 ± 0.18</t>
+          <t>1.27 ± 0.20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABILENE</t>
+          <t>SDN</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CatBoost (Module A)</t>
+          <t>LightGBM (Module A)</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -556,54 +556,54 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.756 ± 0.125</t>
+          <t>5.780 ± 0.793</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[2.661, 2.850]</t>
+          <t>[5.182, 6.377]</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>19.918 ± 7.297</t>
+          <t>39.524 ± 1.102</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[14.416, 25.421]</t>
+          <t>[38.693, 40.355]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.0525 ± 0.0012</t>
+          <t>0.0758 ± 0.0054</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.1493</t>
+          <t>0.0553</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.6016</t>
+          <t>0.2075</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.26 ± 0.33</t>
+          <t>2.65 ± 0.21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABILENE</t>
+          <t>SDN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LightGBM (Module A)</t>
+          <t>LocalSpatialTCN</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -611,54 +611,54 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.908 ± 0.052</t>
+          <t>15.152 ± 0.040</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[2.869, 2.947]</t>
+          <t>[15.122, 15.182]</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>19.854 ± 6.607</t>
+          <t>66.727 ± 0.076</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[14.872, 24.836]</t>
+          <t>[66.670, 66.784]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.0539 ± 0.0005</t>
+          <t>0.1231 ± 0.0002</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.1556</t>
+          <t>0.1451</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.5604</t>
+          <t>0.3050</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.81 ± 0.40</t>
+          <t>1.69 ± 0.22</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABILENE</t>
+          <t>SDN</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LocalSpatialTCN</t>
+          <t>ST-Adaptive-Ensemble (Proposed)</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -666,54 +666,54 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.361 ± 0.000</t>
+          <t>6.562 ± 0.211</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[2.361, 2.362]</t>
+          <t>[6.403, 6.722]</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>17.859 ± 0.001</t>
+          <t>47.268 ± 0.694</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[17.858, 17.860]</t>
+          <t>[46.744, 47.792]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.0486 ± 0.0000</t>
+          <t>0.0810 ± 0.0013</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.1178</t>
+          <t>0.0628</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.2984</t>
+          <t>0.2333</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.52 ± 0.08</t>
+          <t>0.02 ± 0.01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ABILENE</t>
+          <t>SDN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ST-Adaptive-Ensemble (Proposed)</t>
+          <t>ST-WaveFormer</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -721,54 +721,54 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.469 ± 0.474</t>
+          <t>15.350 ± 0.310</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>[2.112, 2.827]</t>
+          <t>[15.117, 15.584]</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>19.741 ± 3.017</t>
+          <t>65.385 ± 1.114</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[17.466, 22.016]</t>
+          <t>[64.545, 66.226]</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.0495 ± 0.0048</t>
+          <t>0.1239 ± 0.0013</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.1232</t>
+          <t>0.1470</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.3907</t>
+          <t>1837.9218</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.00 ± 0.00</t>
+          <t>3.64 ± 0.18</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABILENE</t>
+          <t>SDN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ST-WaveFormer</t>
+          <t>XGBoost (Module A)</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -776,95 +776,700 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.219 ± 0.241</t>
+          <t>5.509 ± 0.031</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[2.038, 2.401]</t>
+          <t>[5.486, 5.532]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>17.177 ± 0.237</t>
+          <t>43.449 ± 0.149</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[16.998, 17.356]</t>
+          <t>[43.336, 43.561]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0.0470 ± 0.0026</t>
+          <t>0.0742 ± 0.0002</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0.1105</t>
+          <t>0.0528</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>3687.1790</t>
+          <t>0.2235</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>3.24 ± 0.11</t>
+          <t>1.98 ± 0.07</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>GEANT</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CatBoost (Module A)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.915 ± 0.003</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[0.912, 0.917]</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>5.902 ± 0.018</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>[5.888, 5.916]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.0302 ± 0.0000</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.1643</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1.6403</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.98 ± 0.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GEANT</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LightGBM (Module A)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.920 ± 0.003</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[0.918, 0.922]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>6.006 ± 0.022</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>[5.990, 6.023]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.0303 ± 0.0000</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.1652</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1.6847</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.98 ± 0.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GEANT</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LocalSpatialTCN</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.854 ± 0.000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[0.854, 0.854]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>5.636 ± 0.002</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>[5.635, 5.637]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.0292 ± 0.0000</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.1534</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1.0706</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1.67 ± 0.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GEANT</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ST-Adaptive-Ensemble (Proposed)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.796 ± 0.025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[0.777, 0.815]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5.481 ± 0.054</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>[5.440, 5.523]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.0282 ± 0.0005</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.1430</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1.2002</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>0.01 ± 0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GEANT</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ST-WaveFormer</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.801 ± 0.063</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[0.753, 0.848]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>5.383 ± 0.013</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>[5.373, 5.392]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.0283 ± 0.0011</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.1438</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2225.1203</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>3.60 ± 0.27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GEANT</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>XGBoost (Module A)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0.915 ± 0.003</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>[0.913, 0.918]</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>5.865 ± 0.014</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>[5.855, 5.875]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.0303 ± 0.0001</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.1644</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1.5777</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>0.76 ± 0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>ABILENE</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CatBoost (Module A)</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2.756 ± 0.125</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>[2.661, 2.850]</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>19.918 ± 7.297</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>[14.416, 25.421]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.0525 ± 0.0012</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0.1493</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>0.6016</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>1.26 ± 0.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ABILENE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LightGBM (Module A)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2.908 ± 0.052</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>[2.869, 2.947]</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>19.854 ± 6.607</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>[14.872, 24.836]</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.0539 ± 0.0005</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.1556</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>0.5604</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>1.81 ± 0.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ABILENE</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LocalSpatialTCN</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2.361 ± 0.000</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>[2.361, 2.362]</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>17.859 ± 0.001</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>[17.858, 17.860]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.0486 ± 0.0000</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.1178</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>0.2984</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>1.52 ± 0.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ABILENE</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ST-Adaptive-Ensemble (Proposed)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2.781 ± 0.993</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>[2.032, 3.529]</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>21.286 ± 5.489</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>[17.147, 25.425]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.0520 ± 0.0088</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>0.1387</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>0.4312</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>0.00 ± 0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ABILENE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ST-WaveFormer</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2.219 ± 0.241</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>[2.038, 2.401]</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>17.177 ± 0.237</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>[16.998, 17.356]</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.0470 ± 0.0026</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0.1105</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>3687.1790</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>3.24 ± 0.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ABILENE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>XGBoost (Module A)</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>2.765 ± 0.012</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>[2.756, 2.774]</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>19.675 ± 6.604</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>[14.696, 24.655]</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>0.0526 ± 0.0001</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>0.1483</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>0.5671</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>1.82 ± 0.41</t>
         </is>

</xml_diff>